<commit_message>
feat: implement custom Application.OnUndo macro for dropdown selections
</commit_message>
<xml_diff>
--- a/reference/列舉定義(企劃用).xlsx
+++ b/reference/列舉定義(企劃用).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AlchemyPlanning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\ExcelEnumSelectionTool\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56080D55-671B-4BB2-A21A-7C37DC8D330F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A85CB4-52FE-461A-A05B-EE3EFD963C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="範例" sheetId="2" r:id="rId1"/>
@@ -161,7 +161,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +199,13 @@
       <family val="2"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -232,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -244,9 +251,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -525,14 +533,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2929DAF4-3B85-4E78-8B94-9EDA6B1D9697}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -540,7 +548,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -551,7 +559,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>29</v>
       </c>
@@ -571,19 +579,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="42.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
     <col min="8" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
@@ -598,7 +606,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -618,7 +626,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -632,7 +640,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -646,7 +654,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -660,7 +668,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -674,7 +682,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="B7" s="7"/>
       <c r="E7" s="1">
         <v>5</v>
       </c>
@@ -682,7 +691,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -690,7 +699,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
@@ -708,7 +717,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -725,7 +734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>2</v>
       </c>
@@ -739,7 +748,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>3</v>
       </c>
@@ -753,7 +762,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>4</v>
       </c>
@@ -761,7 +770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>5</v>
       </c>
@@ -769,7 +778,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>6</v>
       </c>

</xml_diff>